<commit_message>
add fixed navigation bar with leaderboard and profile
</commit_message>
<xml_diff>
--- a/20260621_1.xlsx
+++ b/20260621_1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hobby\MongolNaadam\"/>
@@ -818,6 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -937,6 +938,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="C1:I37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1377,6 +1379,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
@@ -1404,6 +1407,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1460,7 +1464,7 @@
       </c>
       <c r="F2" s="9">
         <f ca="1">+TODAY()</f>
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="G2">
         <f>SUMIF(C:C,E2,B:B)</f>
@@ -1482,7 +1486,7 @@
       </c>
       <c r="F3" s="9">
         <f ca="1">+F2</f>
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G4" si="0">SUMIF(C:C,E3,B:B)</f>
@@ -1504,7 +1508,7 @@
       </c>
       <c r="F4" s="9">
         <f t="shared" ref="F4" ca="1" si="1">+F3</f>
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
@@ -1563,6 +1567,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
new tournament prediction system
</commit_message>
<xml_diff>
--- a/20260621_1.xlsx
+++ b/20260621_1.xlsx
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F2" s="9">
         <f ca="1">+TODAY()</f>
-        <v>46195</v>
+        <v>46198</v>
       </c>
       <c r="G2">
         <f>SUMIF(C:C,E2,B:B)</f>
@@ -1486,7 +1486,7 @@
       </c>
       <c r="F3" s="9">
         <f ca="1">+F2</f>
-        <v>46195</v>
+        <v>46198</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G4" si="0">SUMIF(C:C,E3,B:B)</f>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F4" s="9">
         <f t="shared" ref="F4" ca="1" si="1">+F3</f>
-        <v>46195</v>
+        <v>46198</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
limit picks to max wrestlers per round
</commit_message>
<xml_diff>
--- a/20260621_1.xlsx
+++ b/20260621_1.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="66">
   <si>
     <t>5 давсан бөх</t>
   </si>
@@ -391,6 +391,36 @@
   <si>
     <t>Олгох шагнал</t>
   </si>
+  <si>
+    <t>Нийт орлого</t>
+  </si>
+  <si>
+    <t>Нийт Invest</t>
+  </si>
+  <si>
+    <t>Founder1</t>
+  </si>
+  <si>
+    <t>Invest хугацаа</t>
+  </si>
+  <si>
+    <t>Нийт хүү</t>
+  </si>
+  <si>
+    <t>Нийт Deposit</t>
+  </si>
+  <si>
+    <t>Founder2</t>
+  </si>
+  <si>
+    <t>Founder3</t>
+  </si>
+  <si>
+    <t>Founder4</t>
+  </si>
+  <si>
+    <t>Founder5</t>
+  </si>
 </sst>
 </file>
 
@@ -398,8 +428,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="167" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="[$-409]m/d/yy\ h:mm\ AM/PM;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -495,23 +525,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -522,14 +550,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -537,10 +562,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -874,7 +908,7 @@
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="7" t="s">
         <v>34</v>
       </c>
       <c r="C5" t="s">
@@ -885,7 +919,7 @@
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="7" t="s">
         <v>41</v>
       </c>
       <c r="C6" t="s">
@@ -896,7 +930,7 @@
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>42</v>
       </c>
       <c r="C7" t="s">
@@ -907,7 +941,7 @@
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>43</v>
       </c>
       <c r="C8" t="s">
@@ -918,7 +952,7 @@
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>44</v>
       </c>
       <c r="C9" t="s">
@@ -926,10 +960,10 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B10" s="8"/>
+      <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B11" s="8"/>
+      <c r="B11" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -939,7 +973,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="C1:I37"/>
+  <dimension ref="C1:N37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -949,50 +983,53 @@
     <col min="6" max="6" width="24.44140625" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="3:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="D2" s="5">
+    <row r="2" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="D2" s="4">
         <v>300</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <v>10000</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>3000000</v>
       </c>
     </row>
-    <row r="4" spans="3:6" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="C4" s="2" t="s">
+    <row r="4" spans="3:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="C4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="6" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="D6" s="7" t="s">
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+    </row>
+    <row r="6" spans="3:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>9</v>
       </c>
@@ -1007,7 +1044,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C8" t="s">
         <v>10</v>
       </c>
@@ -1023,7 +1060,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>11</v>
       </c>
@@ -1039,7 +1076,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C10" t="s">
         <v>12</v>
       </c>
@@ -1055,7 +1092,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C11" t="s">
         <v>13</v>
       </c>
@@ -1071,125 +1108,280 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="3:14" x14ac:dyDescent="0.3">
       <c r="F12">
         <f>+SUM(F7:F11)</f>
         <v>202</v>
       </c>
-    </row>
-    <row r="14" spans="3:6" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="C14" s="2" t="s">
+      <c r="L12" s="19">
+        <f>+SUM(L13:L15)</f>
+        <v>108000</v>
+      </c>
+      <c r="M12" s="4">
+        <v>10000</v>
+      </c>
+      <c r="N12">
+        <f>+SUM(N13:N15)</f>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="L13" s="4">
+        <v>100000</v>
+      </c>
+      <c r="M13" s="20">
+        <f>+L13/$L$12</f>
+        <v>0.92592592592592593</v>
+      </c>
+      <c r="N13">
+        <f>+$M$12*M13</f>
+        <v>9259.2592592592591</v>
+      </c>
+    </row>
+    <row r="14" spans="3:14" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="C14" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-    </row>
-    <row r="16" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="D16" s="7" t="s">
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="K14">
+        <f>+J15/K15/24</f>
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="L14" s="4">
+        <v>5000</v>
+      </c>
+      <c r="M14" s="20">
+        <f t="shared" ref="M14:M15" si="1">+L14/$L$12</f>
+        <v>4.6296296296296294E-2</v>
+      </c>
+      <c r="N14">
+        <f t="shared" ref="N14:N15" si="2">+$M$12*M14</f>
+        <v>462.96296296296293</v>
+      </c>
+    </row>
+    <row r="15" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="J15">
+        <v>24</v>
+      </c>
+      <c r="K15">
+        <v>30</v>
+      </c>
+      <c r="L15" s="4">
+        <v>3000</v>
+      </c>
+      <c r="M15" s="20">
+        <f t="shared" si="1"/>
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="2"/>
+        <v>277.77777777777777</v>
+      </c>
+    </row>
+    <row r="16" spans="3:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="5" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="3">
         <f>$F$2/$F$12</f>
         <v>14851.485148514852</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F17" s="3">
         <f>+D17*E17</f>
         <v>14851.485148514852</v>
       </c>
-    </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="K17" s="20">
+        <f>+K21/K20</f>
+        <v>0.2</v>
+      </c>
+      <c r="L17" s="19">
+        <f>+K17*K19</f>
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="18" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C18" t="s">
         <v>1</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="3">
         <f>$F$2/$F$12</f>
         <v>14851.485148514852</v>
       </c>
       <c r="E18">
-        <f>+E17*2</f>
         <v>2</v>
       </c>
-      <c r="F18" s="4">
+      <c r="F18" s="3">
         <f>+D18*E18</f>
         <v>29702.970297029704</v>
       </c>
     </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C19" t="s">
         <v>2</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <f>$F$2/$F$12</f>
         <v>14851.485148514852</v>
       </c>
       <c r="E19">
-        <f t="shared" ref="E19:E21" si="1">+E18*2</f>
-        <v>4</v>
-      </c>
-      <c r="F19" s="4">
+        <v>3</v>
+      </c>
+      <c r="F19" s="3">
         <f>+D19*E19</f>
-        <v>59405.940594059408</v>
-      </c>
-    </row>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.3">
+        <v>44554.455445544554</v>
+      </c>
+      <c r="J19" t="s">
+        <v>56</v>
+      </c>
+      <c r="K19" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="20" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="3">
         <f>$F$2/$F$12</f>
         <v>14851.485148514852</v>
       </c>
       <c r="E20">
-        <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-      <c r="F20" s="4">
+        <v>4</v>
+      </c>
+      <c r="F20" s="3">
         <f>+D20*E20</f>
-        <v>118811.88118811882</v>
-      </c>
-    </row>
-    <row r="21" spans="3:6" x14ac:dyDescent="0.3">
+        <v>59405.940594059408</v>
+      </c>
+      <c r="J20" t="s">
+        <v>57</v>
+      </c>
+      <c r="K20" s="4">
+        <f>+SUM(K21:K25)</f>
+        <v>50000</v>
+      </c>
+      <c r="M20" s="4">
+        <f>+SUM(M21:M25)</f>
+        <v>22833.333333333332</v>
+      </c>
+    </row>
+    <row r="21" spans="3:14" x14ac:dyDescent="0.3">
       <c r="C21" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="3">
         <f>$F$2/$F$12</f>
         <v>14851.485148514852</v>
       </c>
       <c r="E21">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="F21" s="4">
+        <v>5</v>
+      </c>
+      <c r="F21" s="3">
         <f>+D21*E21</f>
-        <v>237623.76237623763</v>
-      </c>
-    </row>
-    <row r="24" spans="3:6" ht="25.8" x14ac:dyDescent="0.5">
-      <c r="C24" s="2" t="s">
+        <v>74257.425742574254</v>
+      </c>
+      <c r="J21" t="s">
+        <v>58</v>
+      </c>
+      <c r="K21" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L21" s="4">
+        <v>1</v>
+      </c>
+      <c r="M21" s="10">
+        <f>+K21/L21</f>
+        <v>10000</v>
+      </c>
+      <c r="N21" s="3"/>
+    </row>
+    <row r="22" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="J22" t="s">
+        <v>62</v>
+      </c>
+      <c r="K22" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L22" s="4">
+        <v>2</v>
+      </c>
+      <c r="M22" s="10">
+        <f t="shared" ref="M22:M25" si="3">+K22/L22</f>
+        <v>5000</v>
+      </c>
+      <c r="N22" s="3"/>
+    </row>
+    <row r="23" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="J23" t="s">
+        <v>63</v>
+      </c>
+      <c r="K23" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L23" s="4">
+        <v>3</v>
+      </c>
+      <c r="M23" s="10">
+        <f t="shared" si="3"/>
+        <v>3333.3333333333335</v>
+      </c>
+      <c r="N23" s="3"/>
+    </row>
+    <row r="24" spans="3:14" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="C24" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="26" spans="3:6" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="D26" s="6" t="s">
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="J24" t="s">
+        <v>64</v>
+      </c>
+      <c r="K24" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L24" s="4">
+        <v>4</v>
+      </c>
+      <c r="M24" s="10">
+        <f t="shared" si="3"/>
+        <v>2500</v>
+      </c>
+      <c r="N24" s="3"/>
+    </row>
+    <row r="25" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="J25" t="s">
+        <v>65</v>
+      </c>
+      <c r="K25" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L25" s="4">
+        <v>5</v>
+      </c>
+      <c r="M25" s="10">
+        <f t="shared" si="3"/>
+        <v>2000</v>
+      </c>
+      <c r="N25" s="3"/>
+    </row>
+    <row r="26" spans="3:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D26" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E26" t="s">
@@ -1199,103 +1391,135 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C27" s="12" t="s">
+    <row r="27" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C27" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D27" s="11">
         <v>1</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E27" s="11">
         <v>4</v>
       </c>
-      <c r="F27" s="12">
+      <c r="F27" s="11">
         <f>+D27*E27</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="28" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C28" s="12" t="s">
+      <c r="J27" t="s">
+        <v>60</v>
+      </c>
+      <c r="K27" s="4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="28" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C28" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="11">
         <f>+D27*2</f>
         <v>2</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E28" s="11">
         <v>2</v>
       </c>
-      <c r="F28" s="12">
-        <f t="shared" ref="F28:F31" si="2">+D28*E28</f>
+      <c r="F28" s="11">
+        <f t="shared" ref="F28:F31" si="4">+D28*E28</f>
         <v>4</v>
       </c>
-    </row>
-    <row r="29" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C29" s="12" t="s">
+      <c r="J28" t="s">
+        <v>61</v>
+      </c>
+      <c r="K28" s="4">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="29" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C29" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D29" s="12">
-        <f t="shared" ref="D29:D31" si="3">+D28*2</f>
+      <c r="D29" s="11">
+        <f t="shared" ref="D29:D31" si="5">+D28*2</f>
         <v>4</v>
       </c>
-      <c r="E29" s="12">
+      <c r="E29" s="11">
         <v>0</v>
       </c>
-      <c r="F29" s="12">
-        <f t="shared" si="2"/>
+      <c r="F29" s="11">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C30" s="12" t="s">
+      <c r="J29" t="s">
+        <v>58</v>
+      </c>
+      <c r="K29" s="4">
+        <v>10000</v>
+      </c>
+      <c r="L29" s="20">
+        <f>+K29/K28</f>
+        <v>0.1</v>
+      </c>
+      <c r="M29" s="19">
+        <f>+L29*K27</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="30" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C30" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="D30" s="12">
-        <f t="shared" si="3"/>
+      <c r="D30" s="11">
+        <f t="shared" si="5"/>
         <v>8</v>
       </c>
-      <c r="E30" s="12">
+      <c r="E30" s="11">
         <v>0</v>
       </c>
-      <c r="F30" s="12">
-        <f t="shared" si="2"/>
+      <c r="F30" s="11">
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C31" s="12" t="s">
+      <c r="J30" t="s">
+        <v>59</v>
+      </c>
+      <c r="K30" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C31" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D31" s="12">
-        <f t="shared" si="3"/>
+      <c r="D31" s="11">
+        <f t="shared" si="5"/>
         <v>16</v>
       </c>
-      <c r="E31" s="12">
+      <c r="E31" s="11">
         <v>1</v>
       </c>
-      <c r="F31" s="12">
-        <f t="shared" si="2"/>
+      <c r="F31" s="11">
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
     </row>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C32" s="13" t="s">
+    <row r="32" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C32" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="12">
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="11">
         <f>+SUM(F27:F31)</f>
         <v>24</v>
       </c>
     </row>
     <row r="33" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="14">
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="12">
         <f>+F17</f>
         <v>14851.485148514852</v>
       </c>
@@ -1305,59 +1529,59 @@
       </c>
       <c r="H33">
         <f>-(F33-E2+G33)*E36</f>
-        <v>-436.63366336633675</v>
-      </c>
-      <c r="I33" s="11">
+        <v>-1746.534653465347</v>
+      </c>
+      <c r="I33" s="10">
         <f>+F33+G33+H33</f>
-        <v>13929.70297029703</v>
+        <v>12619.801980198019</v>
       </c>
     </row>
     <row r="34" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="15">
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="13">
         <f>+F32*F33</f>
         <v>356435.64356435643</v>
       </c>
     </row>
     <row r="35" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C35" s="17" t="s">
+      <c r="C35" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="18"/>
-      <c r="E35" s="16">
+      <c r="D35" s="16"/>
+      <c r="E35" s="14">
         <v>0.1</v>
       </c>
-      <c r="F35" s="14">
+      <c r="F35" s="12">
         <f>-(F34-E2)*E35</f>
         <v>-34643.564356435643</v>
       </c>
     </row>
     <row r="36" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C36" s="17" t="s">
+      <c r="C36" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D36" s="18"/>
-      <c r="E36" s="16">
-        <v>0.1</v>
-      </c>
-      <c r="F36" s="15">
+      <c r="D36" s="16"/>
+      <c r="E36" s="14">
+        <v>0.4</v>
+      </c>
+      <c r="F36" s="13">
         <f>-(F34-E2+F35)*E36</f>
-        <v>-31179.207920792083</v>
+        <v>-124716.83168316833</v>
       </c>
     </row>
     <row r="37" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C37" s="13" t="s">
+      <c r="C37" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="15">
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="13">
         <f>+F34+F36</f>
-        <v>325256.43564356433</v>
+        <v>231718.8118811881</v>
       </c>
     </row>
   </sheetData>
@@ -1450,10 +1674,10 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
+      <c r="A2" s="9">
         <v>46192</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
         <v>1000</v>
       </c>
       <c r="C2" t="s">
@@ -1462,9 +1686,9 @@
       <c r="E2" t="s">
         <v>37</v>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <f ca="1">+TODAY()</f>
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="G2">
         <f>SUMIF(C:C,E2,B:B)</f>
@@ -1472,10 +1696,10 @@
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="10">
+      <c r="A3" s="9">
         <v>46192</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <v>1000</v>
       </c>
       <c r="C3" t="s">
@@ -1484,9 +1708,9 @@
       <c r="E3" t="s">
         <v>38</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="8">
         <f ca="1">+F2</f>
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G4" si="0">SUMIF(C:C,E3,B:B)</f>
@@ -1494,10 +1718,10 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="10">
+      <c r="A4" s="9">
         <v>46192</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <v>1000</v>
       </c>
       <c r="C4" t="s">
@@ -1506,9 +1730,9 @@
       <c r="E4" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="8">
         <f t="shared" ref="F4" ca="1" si="1">+F3</f>
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
@@ -1516,10 +1740,10 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="10">
+      <c r="A5" s="9">
         <v>46193</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="4">
         <v>1000</v>
       </c>
       <c r="C5" t="s">
@@ -1527,10 +1751,10 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A6" s="10">
+      <c r="A6" s="9">
         <v>46193</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="4">
         <v>1000</v>
       </c>
       <c r="C6" t="s">
@@ -1538,10 +1762,10 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" s="10">
+      <c r="A7" s="9">
         <v>46194</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <v>1000</v>
       </c>
       <c r="C7" t="s">
@@ -1549,16 +1773,16 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="5"/>
+      <c r="B9" s="4"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="5"/>
+      <c r="B10" s="4"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="5"/>
+      <c r="B11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>